<commit_message>
refatoração do codigo e melhoramento da lógica existente para melhor fluxo do sistema
</commit_message>
<xml_diff>
--- a/PortoSeguro/Pasta1.xlsx
+++ b/PortoSeguro/Pasta1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kelvi\Downloads\Automacao-Clinica-Odontologica\PortoSeguro\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kelvi\Desktop\AutomaçãoClinica\Automacao-Clinica-Odontologica\PortoSeguro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA7469D-9218-41C0-8BF7-63C462F0F301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542A5836-963D-48A5-A99F-FE4B3018D330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -391,69 +391,45 @@
   <sheetData>
     <row r="1" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
-        <v>32968661</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>32991092</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>32988264</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>32976387</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>32977189</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>32974662</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>32976130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>32938974</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>32919634</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>32953540</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>32867285</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>32919104</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
         <v>32676277</v>
       </c>
     </row>
+    <row r="2" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+    </row>
+    <row r="3" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+    </row>
+    <row r="4" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+    </row>
+    <row r="5" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+    </row>
+    <row r="6" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+    </row>
+    <row r="7" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+    <row r="8" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+    </row>
+    <row r="10" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+    </row>
+    <row r="11" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+    </row>
+    <row r="12" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+    </row>
     <row r="14" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
     </row>
@@ -3316,55 +3292,31 @@
     <row r="967" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A967" s="2"/>
     </row>
-    <row r="968" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A968" s="2"/>
-    </row>
-    <row r="969" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A969" s="2"/>
-    </row>
-    <row r="970" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A970" s="2"/>
-    </row>
-    <row r="971" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A971" s="2"/>
-    </row>
-    <row r="972" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A972" s="2"/>
-    </row>
-    <row r="973" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A973" s="2"/>
-    </row>
-    <row r="974" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A974" s="2"/>
-    </row>
-    <row r="975" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A975" s="2"/>
-    </row>
-    <row r="976" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A976" s="2"/>
-    </row>
-    <row r="977" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A977" s="2"/>
-    </row>
-    <row r="978" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A978" s="2"/>
-    </row>
-    <row r="979" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A979" s="2"/>
-    </row>
-    <row r="980" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="981" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="982" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="983" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="984" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="985" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="986" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="987" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="988" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="989" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="990" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="991" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="992" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>